<commit_message>
Make the error page's suggestions clickable
The failure page told agents to use a toolbar button and to mark the
entry No access; both are now buttons on the page itself, plus Try again.

They work by navigating to a reserved .invalid host that the main process
intercepts and cancels, not through an IPC bridge. The view rendering the
error page is the same one that loads the sites under investigation, so a
preload there would hand that bridge to them. Two guards gate the action:
the view must currently be showing the error document, and the document
navigating must be the local file. Verified in a real BrowserView that
each button fires its action and that a remote page attempting the same
navigation is blocked.

The status write behind No access is factored out of its IPC handler so
both paths share it, and the main window is told to refresh the entry.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/gambling-sites-test.xlsx
+++ b/test-data/gambling-sites-test.xlsx
@@ -125,10 +125,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -160,10 +160,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -441,6 +441,12 @@
       <c r="A3" t="str">
         <v>afhaalchinees.be + derockerbikes.be</v>
       </c>
+      <c r="C3" t="str">
+        <v>Toevoeging zwarte lijst (website + mirrors) + kennisgeving ISP’s | Melding aan DNS BELGIUM</v>
+      </c>
+      <c r="E3" t="str">
+        <v>I086-2026</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2707,6 +2713,9 @@
       <c r="A257" t="str">
         <v>vipluck15.com</v>
       </c>
+      <c r="B257" t="str">
+        <v>No access</v>
+      </c>
       <c r="E257" t="str">
         <v>I019-2026</v>
       </c>
@@ -2725,6 +2734,9 @@
     <row r="259">
       <c r="A259" t="str">
         <v>thorcasino.com</v>
+      </c>
+      <c r="B259" t="str">
+        <v>No access</v>
       </c>
       <c r="E259" t="str">
         <v>I022-2026</v>

</xml_diff>